<commit_message>
feat(resources): add zh variants, input shading + usage hints in Excel
- Add zh-localized copies: pricing-template.zh.xlsx, product-scoring.zh.xlsx,
  ads-sop.zh.md, order-fulfillment-sop.zh.md
- zh page now serves the .zh.* files so Chinese users get native content,
  not the English SOPs
- English Excel sheets now mark input cells yellow and formula cells green,
  plus a one-line 'how to use' under the title
- Fix one size typo (8.0 KB -> 8.7 KB) on the en pricing card
</commit_message>
<xml_diff>
--- a/public/downloads/pricing-template.xlsx
+++ b/public/downloads/pricing-template.xlsx
@@ -22,7 +22,7 @@
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
     <numFmt numFmtId="165" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="6">
+  <fonts count="8">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -40,6 +40,14 @@
     </font>
     <font>
       <b val="1"/>
+      <color rgb="00B7791F"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="002F855A"/>
+    </font>
+    <font>
+      <b val="1"/>
       <color rgb="00FFFFFF"/>
     </font>
     <font>
@@ -50,12 +58,22 @@
       <sz val="12"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FEF3C7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C6F6D5"/>
+      </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -85,30 +103,33 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -477,7 +498,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q7"/>
+  <dimension ref="A1:Q12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -491,6 +512,7 @@
     <col width="12" customWidth="1" min="9" max="9"/>
     <col width="12" customWidth="1" min="10" max="10"/>
     <col width="32" customWidth="1" min="11" max="11"/>
+    <col width="3" customWidth="1" min="12" max="12"/>
     <col width="13" customWidth="1" min="13" max="13"/>
     <col width="13" customWidth="1" min="14" max="14"/>
     <col width="14" customWidth="1" min="15" max="15"/>
@@ -508,273 +530,442 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Fill in B/C/D/... cells. Read-only formulas in M–P. Currency: USD.</t>
+          <t>Yellow cells = your inputs. Gray cells = auto-calculated. Do not type into gray cells.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>↓ Inputs ↓</t>
+        </is>
+      </c>
+      <c r="L3" s="4" t="inlineStr">
+        <is>
+          <t>↓ Formulas (read-only) ↓</t>
         </is>
       </c>
     </row>
     <row r="4" ht="32" customHeight="1">
-      <c r="A4" s="3" t="inlineStr">
+      <c r="A4" s="5" t="inlineStr">
         <is>
           <t>SKU</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B4" s="5" t="inlineStr">
         <is>
           <t>COGS</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="C4" s="5" t="inlineStr">
         <is>
           <t>Inbound (per unit)</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="D4" s="5" t="inlineStr">
         <is>
           <t>Outbound (per unit)</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="E4" s="5" t="inlineStr">
         <is>
           <t>Platform fee %</t>
         </is>
       </c>
-      <c r="F4" s="3" t="inlineStr">
+      <c r="F4" s="5" t="inlineStr">
         <is>
           <t>Payment fee %</t>
         </is>
       </c>
-      <c r="G4" s="3" t="inlineStr">
+      <c r="G4" s="5" t="inlineStr">
         <is>
           <t>Target margin %</t>
         </is>
       </c>
-      <c r="H4" s="3" t="inlineStr">
+      <c r="H4" s="5" t="inlineStr">
         <is>
           <t>Refund reserve %</t>
         </is>
       </c>
-      <c r="I4" s="3" t="inlineStr">
+      <c r="I4" s="5" t="inlineStr">
         <is>
           <t>Ad % of revenue</t>
         </is>
       </c>
-      <c r="J4" s="3" t="inlineStr">
+      <c r="J4" s="5" t="inlineStr">
         <is>
           <t>Other fixed cost</t>
         </is>
       </c>
-      <c r="K4" s="3" t="inlineStr">
+      <c r="K4" s="5" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
-      <c r="M4" s="4" t="inlineStr">
+      <c r="M4" s="6" t="inlineStr">
         <is>
           <t>Sum cost/unit</t>
         </is>
       </c>
-      <c r="N4" s="4" t="inlineStr">
+      <c r="N4" s="6" t="inlineStr">
         <is>
           <t>Variable cost %</t>
         </is>
       </c>
-      <c r="O4" s="4" t="inlineStr">
+      <c r="O4" s="6" t="inlineStr">
         <is>
           <t>Suggested price</t>
         </is>
       </c>
-      <c r="P4" s="4" t="inlineStr">
+      <c r="P4" s="6" t="inlineStr">
         <is>
           <t>Break-even price</t>
         </is>
       </c>
-      <c r="Q4" s="4" t="inlineStr">
+      <c r="Q4" s="6" t="inlineStr">
         <is>
           <t>Net profit/unit</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="5" t="inlineStr">
+      <c r="A5" s="7" t="inlineStr">
         <is>
           <t>SKU-001</t>
         </is>
       </c>
-      <c r="B5" s="6" t="n">
+      <c r="B5" s="8" t="n">
         <v>4.5</v>
       </c>
-      <c r="C5" s="6" t="n">
+      <c r="C5" s="8" t="n">
         <v>1.2</v>
       </c>
-      <c r="D5" s="6" t="n">
+      <c r="D5" s="8" t="n">
         <v>3.8</v>
       </c>
-      <c r="E5" s="6" t="n">
+      <c r="E5" s="8" t="n">
         <v>0.06</v>
       </c>
-      <c r="F5" s="6" t="n">
+      <c r="F5" s="8" t="n">
         <v>0.029</v>
       </c>
-      <c r="G5" s="6" t="n">
+      <c r="G5" s="8" t="n">
         <v>0.25</v>
       </c>
-      <c r="H5" s="6" t="n">
+      <c r="H5" s="8" t="n">
         <v>0.03</v>
       </c>
-      <c r="I5" s="6" t="n">
+      <c r="I5" s="8" t="n">
         <v>0.15</v>
       </c>
-      <c r="J5" s="6" t="n">
+      <c r="J5" s="8" t="n">
         <v>0.1</v>
       </c>
-      <c r="K5" s="7" t="inlineStr">
+      <c r="K5" s="9" t="inlineStr">
         <is>
           <t>Wireless earbuds, AliExpress → US</t>
         </is>
       </c>
-      <c r="M5" s="8">
+      <c r="M5" s="10">
         <f>B5+C5+D5+J5</f>
         <v/>
       </c>
-      <c r="N5" s="9">
+      <c r="N5" s="11">
         <f>E5+F5+H5+I5</f>
         <v/>
       </c>
-      <c r="O5" s="8">
+      <c r="O5" s="10">
         <f>IFERROR(M5/(1-N5-G5),0)</f>
         <v/>
       </c>
-      <c r="P5" s="8">
+      <c r="P5" s="10">
         <f>IFERROR(M5/(1-N5),0)</f>
         <v/>
       </c>
-      <c r="Q5" s="8">
+      <c r="Q5" s="10">
         <f>O5-M5-O5*N5</f>
         <v/>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="5" t="inlineStr">
+      <c r="A6" s="7" t="inlineStr">
         <is>
           <t>SKU-002</t>
         </is>
       </c>
-      <c r="B6" s="6" t="n">
+      <c r="B6" s="8" t="n">
         <v>7.8</v>
       </c>
-      <c r="C6" s="6" t="n">
+      <c r="C6" s="8" t="n">
         <v>1.5</v>
       </c>
-      <c r="D6" s="6" t="n">
+      <c r="D6" s="8" t="n">
         <v>4.2</v>
       </c>
-      <c r="E6" s="6" t="n">
+      <c r="E6" s="8" t="n">
         <v>0.06</v>
       </c>
-      <c r="F6" s="6" t="n">
+      <c r="F6" s="8" t="n">
         <v>0.029</v>
       </c>
-      <c r="G6" s="6" t="n">
+      <c r="G6" s="8" t="n">
         <v>0.3</v>
       </c>
-      <c r="H6" s="6" t="n">
+      <c r="H6" s="8" t="n">
         <v>0.04</v>
       </c>
-      <c r="I6" s="6" t="n">
+      <c r="I6" s="8" t="n">
         <v>0.2</v>
       </c>
-      <c r="J6" s="6" t="n">
+      <c r="J6" s="8" t="n">
         <v>0.2</v>
       </c>
-      <c r="K6" s="7" t="inlineStr">
+      <c r="K6" s="9" t="inlineStr">
         <is>
           <t>Phone case, China Post e-packet</t>
         </is>
       </c>
-      <c r="M6" s="8">
+      <c r="M6" s="10">
         <f>B6+C6+D6+J6</f>
         <v/>
       </c>
-      <c r="N6" s="9">
+      <c r="N6" s="11">
         <f>E6+F6+H6+I6</f>
         <v/>
       </c>
-      <c r="O6" s="8">
+      <c r="O6" s="10">
         <f>IFERROR(M6/(1-N6-G6),0)</f>
         <v/>
       </c>
-      <c r="P6" s="8">
+      <c r="P6" s="10">
         <f>IFERROR(M6/(1-N6),0)</f>
         <v/>
       </c>
-      <c r="Q6" s="8">
+      <c r="Q6" s="10">
         <f>O6-M6-O6*N6</f>
         <v/>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="5" t="inlineStr">
+      <c r="A7" s="7" t="inlineStr">
         <is>
           <t>SKU-003</t>
         </is>
       </c>
-      <c r="B7" s="6" t="n">
+      <c r="B7" s="8" t="n">
         <v>2.1</v>
       </c>
-      <c r="C7" s="6" t="n">
+      <c r="C7" s="8" t="n">
         <v>0.9</v>
       </c>
-      <c r="D7" s="6" t="n">
+      <c r="D7" s="8" t="n">
         <v>2.6</v>
       </c>
-      <c r="E7" s="6" t="n">
+      <c r="E7" s="8" t="n">
         <v>0.1</v>
       </c>
-      <c r="F7" s="6" t="n">
+      <c r="F7" s="8" t="n">
         <v>0.029</v>
       </c>
-      <c r="G7" s="6" t="n">
+      <c r="G7" s="8" t="n">
         <v>0.2</v>
       </c>
-      <c r="H7" s="6" t="n">
+      <c r="H7" s="8" t="n">
         <v>0.05</v>
       </c>
-      <c r="I7" s="6" t="n">
+      <c r="I7" s="8" t="n">
         <v>0.1</v>
       </c>
-      <c r="J7" s="6" t="n">
+      <c r="J7" s="8" t="n">
         <v>0.05</v>
       </c>
-      <c r="K7" s="7" t="inlineStr">
+      <c r="K7" s="9" t="inlineStr">
         <is>
           <t>Bestseller T-shirt, FBA</t>
         </is>
       </c>
-      <c r="M7" s="8">
+      <c r="M7" s="10">
         <f>B7+C7+D7+J7</f>
         <v/>
       </c>
-      <c r="N7" s="9">
+      <c r="N7" s="11">
         <f>E7+F7+H7+I7</f>
         <v/>
       </c>
-      <c r="O7" s="8">
+      <c r="O7" s="10">
         <f>IFERROR(M7/(1-N7-G7),0)</f>
         <v/>
       </c>
-      <c r="P7" s="8">
+      <c r="P7" s="10">
         <f>IFERROR(M7/(1-N7),0)</f>
         <v/>
       </c>
-      <c r="Q7" s="8">
+      <c r="Q7" s="10">
         <f>O7-M7-O7*N7</f>
         <v/>
       </c>
     </row>
+    <row r="8">
+      <c r="B8" s="12" t="n"/>
+      <c r="C8" s="12" t="n"/>
+      <c r="D8" s="12" t="n"/>
+      <c r="E8" s="12" t="n"/>
+      <c r="F8" s="12" t="n"/>
+      <c r="G8" s="12" t="n"/>
+      <c r="H8" s="12" t="n"/>
+      <c r="I8" s="12" t="n"/>
+      <c r="J8" s="12" t="n"/>
+      <c r="M8" s="10">
+        <f>B8+C8+D8+J8</f>
+        <v/>
+      </c>
+      <c r="N8" s="11">
+        <f>E8+F8+H8+I8</f>
+        <v/>
+      </c>
+      <c r="O8" s="10">
+        <f>IFERROR(M8/(1-N8-G8),0)</f>
+        <v/>
+      </c>
+      <c r="P8" s="10">
+        <f>IFERROR(M8/(1-N8),0)</f>
+        <v/>
+      </c>
+      <c r="Q8" s="10">
+        <f>O8-M8-O8*N8</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="B9" s="12" t="n"/>
+      <c r="C9" s="12" t="n"/>
+      <c r="D9" s="12" t="n"/>
+      <c r="E9" s="12" t="n"/>
+      <c r="F9" s="12" t="n"/>
+      <c r="G9" s="12" t="n"/>
+      <c r="H9" s="12" t="n"/>
+      <c r="I9" s="12" t="n"/>
+      <c r="J9" s="12" t="n"/>
+      <c r="M9" s="10">
+        <f>B9+C9+D9+J9</f>
+        <v/>
+      </c>
+      <c r="N9" s="11">
+        <f>E9+F9+H9+I9</f>
+        <v/>
+      </c>
+      <c r="O9" s="10">
+        <f>IFERROR(M9/(1-N9-G9),0)</f>
+        <v/>
+      </c>
+      <c r="P9" s="10">
+        <f>IFERROR(M9/(1-N9),0)</f>
+        <v/>
+      </c>
+      <c r="Q9" s="10">
+        <f>O9-M9-O9*N9</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="B10" s="12" t="n"/>
+      <c r="C10" s="12" t="n"/>
+      <c r="D10" s="12" t="n"/>
+      <c r="E10" s="12" t="n"/>
+      <c r="F10" s="12" t="n"/>
+      <c r="G10" s="12" t="n"/>
+      <c r="H10" s="12" t="n"/>
+      <c r="I10" s="12" t="n"/>
+      <c r="J10" s="12" t="n"/>
+      <c r="M10" s="10">
+        <f>B10+C10+D10+J10</f>
+        <v/>
+      </c>
+      <c r="N10" s="11">
+        <f>E10+F10+H10+I10</f>
+        <v/>
+      </c>
+      <c r="O10" s="10">
+        <f>IFERROR(M10/(1-N10-G10),0)</f>
+        <v/>
+      </c>
+      <c r="P10" s="10">
+        <f>IFERROR(M10/(1-N10),0)</f>
+        <v/>
+      </c>
+      <c r="Q10" s="10">
+        <f>O10-M10-O10*N10</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="B11" s="12" t="n"/>
+      <c r="C11" s="12" t="n"/>
+      <c r="D11" s="12" t="n"/>
+      <c r="E11" s="12" t="n"/>
+      <c r="F11" s="12" t="n"/>
+      <c r="G11" s="12" t="n"/>
+      <c r="H11" s="12" t="n"/>
+      <c r="I11" s="12" t="n"/>
+      <c r="J11" s="12" t="n"/>
+      <c r="M11" s="10">
+        <f>B11+C11+D11+J11</f>
+        <v/>
+      </c>
+      <c r="N11" s="11">
+        <f>E11+F11+H11+I11</f>
+        <v/>
+      </c>
+      <c r="O11" s="10">
+        <f>IFERROR(M11/(1-N11-G11),0)</f>
+        <v/>
+      </c>
+      <c r="P11" s="10">
+        <f>IFERROR(M11/(1-N11),0)</f>
+        <v/>
+      </c>
+      <c r="Q11" s="10">
+        <f>O11-M11-O11*N11</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="B12" s="12" t="n"/>
+      <c r="C12" s="12" t="n"/>
+      <c r="D12" s="12" t="n"/>
+      <c r="E12" s="12" t="n"/>
+      <c r="F12" s="12" t="n"/>
+      <c r="G12" s="12" t="n"/>
+      <c r="H12" s="12" t="n"/>
+      <c r="I12" s="12" t="n"/>
+      <c r="J12" s="12" t="n"/>
+      <c r="M12" s="10">
+        <f>B12+C12+D12+J12</f>
+        <v/>
+      </c>
+      <c r="N12" s="11">
+        <f>E12+F12+H12+I12</f>
+        <v/>
+      </c>
+      <c r="O12" s="10">
+        <f>IFERROR(M12/(1-N12-G12),0)</f>
+        <v/>
+      </c>
+      <c r="P12" s="10">
+        <f>IFERROR(M12/(1-N12),0)</f>
+        <v/>
+      </c>
+      <c r="Q12" s="10">
+        <f>O12-M12-O12*N12</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="A2:K2"/>
-    <mergeCell ref="A1:K1"/>
+  <mergeCells count="4">
+    <mergeCell ref="A2:Q2"/>
+    <mergeCell ref="A1:Q1"/>
+    <mergeCell ref="L3:Q3"/>
+    <mergeCell ref="A3:K3"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -786,7 +977,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B12"/>
+  <dimension ref="A1:B13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -794,19 +985,19 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="10" t="inlineStr">
+      <c r="A1" s="13" t="inlineStr">
         <is>
           <t>Field</t>
         </is>
       </c>
-      <c r="B1" s="10" t="inlineStr">
+      <c r="B1" s="13" t="inlineStr">
         <is>
           <t>Meaning</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="11" t="inlineStr">
+      <c r="A2" s="14" t="inlineStr">
         <is>
           <t>COGS</t>
         </is>
@@ -818,7 +1009,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="11" t="inlineStr">
+      <c r="A3" s="14" t="inlineStr">
         <is>
           <t>Inbound</t>
         </is>
@@ -830,7 +1021,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="11" t="inlineStr">
+      <c r="A4" s="14" t="inlineStr">
         <is>
           <t>Outbound</t>
         </is>
@@ -842,7 +1033,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="11" t="inlineStr">
+      <c r="A5" s="14" t="inlineStr">
         <is>
           <t>Platform fee %</t>
         </is>
@@ -854,7 +1045,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="11" t="inlineStr">
+      <c r="A6" s="14" t="inlineStr">
         <is>
           <t>Payment fee %</t>
         </is>
@@ -866,7 +1057,7 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="11" t="inlineStr">
+      <c r="A7" s="14" t="inlineStr">
         <is>
           <t>Target margin %</t>
         </is>
@@ -878,7 +1069,7 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="11" t="inlineStr">
+      <c r="A8" s="14" t="inlineStr">
         <is>
           <t>Refund reserve %</t>
         </is>
@@ -890,7 +1081,7 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="11" t="inlineStr">
+      <c r="A9" s="14" t="inlineStr">
         <is>
           <t>Ad % of revenue</t>
         </is>
@@ -902,7 +1093,7 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="11" t="inlineStr">
+      <c r="A10" s="14" t="inlineStr">
         <is>
           <t>Other fixed cost</t>
         </is>
@@ -914,7 +1105,7 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="11" t="inlineStr">
+      <c r="A11" s="14" t="inlineStr">
         <is>
           <t>Suggested price</t>
         </is>
@@ -926,7 +1117,7 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="11" t="inlineStr">
+      <c r="A12" s="14" t="inlineStr">
         <is>
           <t>Break-even price</t>
         </is>
@@ -934,6 +1125,18 @@
       <c r="B12" t="inlineStr">
         <is>
           <t>Price at which net profit = 0.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="14" t="inlineStr">
+        <is>
+          <t>Net profit / unit</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Suggested price − all costs including variable %.</t>
         </is>
       </c>
     </row>
@@ -955,63 +1158,63 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="12" t="inlineStr">
+      <c r="A1" s="15" t="inlineStr">
         <is>
           <t>What this template does NOT cover</t>
         </is>
       </c>
     </row>
     <row r="3" ht="36" customHeight="1">
-      <c r="A3" s="13" t="inlineStr">
+      <c r="A3" s="16" t="inlineStr">
         <is>
           <t>• FX conversion. All numbers in USD. If your revenue is in EUR/GBP, convert at the rate you actually receive (after FX margin).</t>
         </is>
       </c>
     </row>
     <row r="4" ht="36" customHeight="1">
-      <c r="A4" s="13" t="inlineStr">
+      <c r="A4" s="16" t="inlineStr">
         <is>
           <t>• Inventory carrying cost. Add if you hold &gt; 60 days of stock.</t>
         </is>
       </c>
     </row>
     <row r="5" ht="36" customHeight="1">
-      <c r="A5" s="13" t="inlineStr">
+      <c r="A5" s="16" t="inlineStr">
         <is>
           <t>• Returns logistics cost. Refund reserve % is revenue-side; add return shipping as a separate per-unit cost.</t>
         </is>
       </c>
     </row>
     <row r="6" ht="36" customHeight="1">
-      <c r="A6" s="13" t="inlineStr">
+      <c r="A6" s="16" t="inlineStr">
         <is>
           <t>• Tax. Sales tax / VAT not subtracted here. Apply separately on the suggested price.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="36" customHeight="1">
-      <c r="A7" s="13" t="inlineStr">
+      <c r="A7" s="16" t="inlineStr">
         <is>
           <t>• Subscription / SaaS tools (Klaviyo, AppSumo apps). Add as monthly fixed ÷ monthly units.</t>
         </is>
       </c>
     </row>
     <row r="8" ht="36" customHeight="1">
-      <c r="A8" s="13" t="inlineStr">
+      <c r="A8" s="16" t="inlineStr">
         <is>
           <t>• Per-SKU shipping discount tiers. Outbound cost should already reflect negotiated rates.</t>
         </is>
       </c>
     </row>
     <row r="9" ht="36" customHeight="1">
-      <c r="A9" s="13" t="inlineStr">
+      <c r="A9" s="16" t="inlineStr">
         <is>
           <t>• Promo / discount campaigns. If you run 20% off, the realized price is O * 0.8; rerun the formula at the new price.</t>
         </is>
       </c>
     </row>
     <row r="10" ht="36" customHeight="1">
-      <c r="A10" s="13" t="inlineStr">
+      <c r="A10" s="16" t="inlineStr">
         <is>
           <t>• Break-even is unit economics only. Cash-flow break-even requires working-capital timing.</t>
         </is>

</xml_diff>